<commit_message>
state: bot run 2026-09-04T19:49 IST
</commit_message>
<xml_diff>
--- a/data/trade_log_india.xlsx
+++ b/data/trade_log_india.xlsx
@@ -431,61 +431,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Close</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>SMA20</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Upper_Band</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>EMA9</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>EMA21</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Vol_Ratio</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Qualifies</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Rejection_Or_Status</t>
         </is>
@@ -1047,6 +1047,547 @@
       <c r="K14" t="inlineStr">
         <is>
           <t>BELOW_BAND (Close 1325.50 &lt;= Upper 1339.41)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>19:49:24</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>TRENT</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>2853</v>
+      </c>
+      <c r="E15" t="n">
+        <v>3039.71</v>
+      </c>
+      <c r="F15" t="n">
+        <v>3039.71</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2871.99</v>
+      </c>
+      <c r="H15" t="n">
+        <v>2912.6</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="J15" t="b">
+        <v>0</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2871.99 &lt;= EMA21 2912.60)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>19:49:24</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="J16" t="b">
+        <v>0</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_DATA (&lt; 30 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>19:49:24</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>HAL</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>4856</v>
+      </c>
+      <c r="E17" t="n">
+        <v>5109.33</v>
+      </c>
+      <c r="F17" t="n">
+        <v>5109.33</v>
+      </c>
+      <c r="G17" t="n">
+        <v>4841.36</v>
+      </c>
+      <c r="H17" t="n">
+        <v>4841.16</v>
+      </c>
+      <c r="I17" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="J17" t="b">
+        <v>0</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 4856.00 &lt;= Upper 5109.33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>19:49:24</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>PERSISTENT</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>5643</v>
+      </c>
+      <c r="E18" t="n">
+        <v>5832.9</v>
+      </c>
+      <c r="F18" t="n">
+        <v>5832.9</v>
+      </c>
+      <c r="G18" t="n">
+        <v>5670.08</v>
+      </c>
+      <c r="H18" t="n">
+        <v>5597.1</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="J18" t="b">
+        <v>0</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 5643.00 &lt;= Upper 5832.90)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>19:49:24</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>DIXON</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>14240</v>
+      </c>
+      <c r="E19" t="n">
+        <v>15129.44</v>
+      </c>
+      <c r="F19" t="n">
+        <v>15129.44</v>
+      </c>
+      <c r="G19" t="n">
+        <v>14513.77</v>
+      </c>
+      <c r="H19" t="n">
+        <v>14411.98</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J19" t="b">
+        <v>0</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 14240.00 &lt;= Upper 15129.44)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>19:49:24</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1840</v>
+      </c>
+      <c r="E20" t="n">
+        <v>2004.05</v>
+      </c>
+      <c r="F20" t="n">
+        <v>2004.05</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1873.89</v>
+      </c>
+      <c r="H20" t="n">
+        <v>1898.48</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="J20" t="b">
+        <v>0</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1873.89 &lt;= EMA21 1898.48)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>19:49:24</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>MCX</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>3275.4</v>
+      </c>
+      <c r="E21" t="n">
+        <v>3507.94</v>
+      </c>
+      <c r="F21" t="n">
+        <v>3507.94</v>
+      </c>
+      <c r="G21" t="n">
+        <v>3247.81</v>
+      </c>
+      <c r="H21" t="n">
+        <v>3132.48</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="J21" t="b">
+        <v>0</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 3275.40 &lt;= Upper 3507.94)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>19:49:24</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1839</v>
+      </c>
+      <c r="E22" t="n">
+        <v>1935.31</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1935.31</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1848.54</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1853.3</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J22" t="b">
+        <v>0</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1848.54 &lt;= EMA21 1853.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>19:49:24</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>712.1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>739.1799999999999</v>
+      </c>
+      <c r="F23" t="n">
+        <v>739.1799999999999</v>
+      </c>
+      <c r="G23" t="n">
+        <v>713.23</v>
+      </c>
+      <c r="H23" t="n">
+        <v>723.11</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="J23" t="b">
+        <v>0</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 713.23 &lt;= EMA21 723.11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>19:49:24</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1423.2</v>
+      </c>
+      <c r="E24" t="n">
+        <v>1449.22</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1449.22</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1429.18</v>
+      </c>
+      <c r="H24" t="n">
+        <v>1426.22</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J24" t="b">
+        <v>0</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1423.20 &lt;= Upper 1449.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>19:49:24</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>POLYCAB</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>8300</v>
+      </c>
+      <c r="E25" t="n">
+        <v>9580.41</v>
+      </c>
+      <c r="F25" t="n">
+        <v>9580.41</v>
+      </c>
+      <c r="G25" t="n">
+        <v>8862.83</v>
+      </c>
+      <c r="H25" t="n">
+        <v>9011.360000000001</v>
+      </c>
+      <c r="I25" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="J25" t="b">
+        <v>0</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 8862.83 &lt;= EMA21 9011.36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>19:49:24</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>VBL</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>407.6</v>
+      </c>
+      <c r="E26" t="n">
+        <v>454.24</v>
+      </c>
+      <c r="F26" t="n">
+        <v>454.24</v>
+      </c>
+      <c r="G26" t="n">
+        <v>413.95</v>
+      </c>
+      <c r="H26" t="n">
+        <v>425.31</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J26" t="b">
+        <v>0</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 413.95 &lt;= EMA21 425.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>19:49:24</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1322</v>
+      </c>
+      <c r="E27" t="n">
+        <v>1338.89</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1338.89</v>
+      </c>
+      <c r="G27" t="n">
+        <v>1306.11</v>
+      </c>
+      <c r="H27" t="n">
+        <v>1306</v>
+      </c>
+      <c r="I27" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="J27" t="b">
+        <v>0</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1322.00 &lt;= Upper 1338.89)</t>
         </is>
       </c>
     </row>
@@ -1116,57 +1657,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Entry_Date</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Entry_Price</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Invested</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Current_Price</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Unrealized_PnL_Pct</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Hard_SL</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Highest_High</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Days_Held</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -1187,67 +1728,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Entry_Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Exit_Date</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Entry_Price</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Exit_Price</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Invested</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Gross_PnL_Pct</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Net_PnL_Pct</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>PnL_Amount</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Exit_Reason</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Days_Held</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -1982,57 +2523,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Order_ID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Side</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Expected_Price</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Fill_Price</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Slippage</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -7037,27 +7578,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
@@ -7101,51 +7642,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cash_Available</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Invested_Capital</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Total_Equity</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Realized_PnL</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Win_Rate_Pct</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Total_Trades</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Open_Positions</t>
         </is>
@@ -7181,6 +7722,39 @@
         <v>17</v>
       </c>
       <c r="I2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>19:49:24</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>198821.93</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>198821.93</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>17</v>
+      </c>
+      <c r="I3" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update trade_log_india.xlsx with realized pnl
</commit_message>
<xml_diff>
--- a/data/trade_log_india.xlsx
+++ b/data/trade_log_india.xlsx
@@ -431,61 +431,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Close</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>SMA20</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Upper_Band</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>EMA9</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>EMA21</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Vol_Ratio</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Qualifies</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Rejection_Or_Status</t>
         </is>
@@ -1586,6 +1586,565 @@
         <v>0</v>
       </c>
       <c r="K27" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1322.00 &lt;= Upper 1338.89)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>12:57:48</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>TRENT</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>2815.6</v>
+      </c>
+      <c r="E28" t="n">
+        <v>3046.08</v>
+      </c>
+      <c r="F28" t="n">
+        <v>3046.08</v>
+      </c>
+      <c r="G28" t="n">
+        <v>2876.74</v>
+      </c>
+      <c r="H28" t="n">
+        <v>2918.56</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="J28" t="b">
+        <v>0</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2876.74 &lt;= EMA21 2918.56)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>12:57:48</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>405.35</v>
+      </c>
+      <c r="E29" t="n">
+        <v>415.92</v>
+      </c>
+      <c r="F29" t="n">
+        <v>415.92</v>
+      </c>
+      <c r="G29" t="n">
+        <v>408.81</v>
+      </c>
+      <c r="H29" t="n">
+        <v>408.04</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="J29" t="b">
+        <v>0</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 405.35 &lt;= Upper 415.92)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>12:57:48</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>HAL</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>4856</v>
+      </c>
+      <c r="E30" t="n">
+        <v>5109.33</v>
+      </c>
+      <c r="F30" t="n">
+        <v>5109.33</v>
+      </c>
+      <c r="G30" t="n">
+        <v>4841.36</v>
+      </c>
+      <c r="H30" t="n">
+        <v>4841.16</v>
+      </c>
+      <c r="I30" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="J30" t="b">
+        <v>0</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 4856.00 &lt;= Upper 5109.33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>12:57:48</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>PERSISTENT</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>5643</v>
+      </c>
+      <c r="E31" t="n">
+        <v>5832.9</v>
+      </c>
+      <c r="F31" t="n">
+        <v>5832.9</v>
+      </c>
+      <c r="G31" t="n">
+        <v>5670.08</v>
+      </c>
+      <c r="H31" t="n">
+        <v>5597.1</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="J31" t="b">
+        <v>0</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 5643.00 &lt;= Upper 5832.90)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>12:57:48</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>DIXON</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>14445</v>
+      </c>
+      <c r="E32" t="n">
+        <v>15130.01</v>
+      </c>
+      <c r="F32" t="n">
+        <v>15130.01</v>
+      </c>
+      <c r="G32" t="n">
+        <v>14582.21</v>
+      </c>
+      <c r="H32" t="n">
+        <v>14429.18</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J32" t="b">
+        <v>0</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 14445.00 &lt;= Upper 15130.01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>12:57:48</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1840</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2004.05</v>
+      </c>
+      <c r="F33" t="n">
+        <v>2004.05</v>
+      </c>
+      <c r="G33" t="n">
+        <v>1873.89</v>
+      </c>
+      <c r="H33" t="n">
+        <v>1898.48</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="J33" t="b">
+        <v>0</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1873.89 &lt;= EMA21 1898.48)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>12:57:48</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>MCX</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>3275.4</v>
+      </c>
+      <c r="E34" t="n">
+        <v>3507.94</v>
+      </c>
+      <c r="F34" t="n">
+        <v>3507.94</v>
+      </c>
+      <c r="G34" t="n">
+        <v>3247.81</v>
+      </c>
+      <c r="H34" t="n">
+        <v>3132.48</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="J34" t="b">
+        <v>0</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 3275.40 &lt;= Upper 3507.94)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>12:57:48</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>1839</v>
+      </c>
+      <c r="E35" t="n">
+        <v>1935.31</v>
+      </c>
+      <c r="F35" t="n">
+        <v>1935.31</v>
+      </c>
+      <c r="G35" t="n">
+        <v>1848.54</v>
+      </c>
+      <c r="H35" t="n">
+        <v>1853.3</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J35" t="b">
+        <v>0</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1848.54 &lt;= EMA21 1853.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>12:57:48</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>712.1</v>
+      </c>
+      <c r="E36" t="n">
+        <v>739.1799999999999</v>
+      </c>
+      <c r="F36" t="n">
+        <v>739.1799999999999</v>
+      </c>
+      <c r="G36" t="n">
+        <v>713.23</v>
+      </c>
+      <c r="H36" t="n">
+        <v>723.11</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="J36" t="b">
+        <v>0</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 713.23 &lt;= EMA21 723.11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>12:57:48</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>1423.2</v>
+      </c>
+      <c r="E37" t="n">
+        <v>1449.22</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1449.22</v>
+      </c>
+      <c r="G37" t="n">
+        <v>1429.18</v>
+      </c>
+      <c r="H37" t="n">
+        <v>1426.22</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J37" t="b">
+        <v>0</v>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1423.20 &lt;= Upper 1449.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>12:57:48</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>POLYCAB</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>8300</v>
+      </c>
+      <c r="E38" t="n">
+        <v>9580.41</v>
+      </c>
+      <c r="F38" t="n">
+        <v>9580.41</v>
+      </c>
+      <c r="G38" t="n">
+        <v>8862.83</v>
+      </c>
+      <c r="H38" t="n">
+        <v>9011.360000000001</v>
+      </c>
+      <c r="I38" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="J38" t="b">
+        <v>0</v>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 8862.83 &lt;= EMA21 9011.36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>12:57:48</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>VBL</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>407.6</v>
+      </c>
+      <c r="E39" t="n">
+        <v>454.24</v>
+      </c>
+      <c r="F39" t="n">
+        <v>454.24</v>
+      </c>
+      <c r="G39" t="n">
+        <v>413.95</v>
+      </c>
+      <c r="H39" t="n">
+        <v>425.31</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J39" t="b">
+        <v>0</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 413.95 &lt;= EMA21 425.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>12:57:48</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>1322</v>
+      </c>
+      <c r="E40" t="n">
+        <v>1338.89</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1338.89</v>
+      </c>
+      <c r="G40" t="n">
+        <v>1306.11</v>
+      </c>
+      <c r="H40" t="n">
+        <v>1306</v>
+      </c>
+      <c r="I40" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="J40" t="b">
+        <v>0</v>
+      </c>
+      <c r="K40" t="inlineStr">
         <is>
           <t>BELOW_BAND (Close 1322.00 &lt;= Upper 1338.89)</t>
         </is>
@@ -1657,57 +2216,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Entry_Date</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Entry_Price</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Invested</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Current_Price</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Unrealized_PnL_Pct</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Hard_SL</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Highest_High</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Days_Held</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -1728,67 +2287,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Entry_Date</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Exit_Date</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Entry_Price</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Exit_Price</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Invested</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Gross_PnL_Pct</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Net_PnL_Pct</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>PnL_Amount</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Exit_Reason</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Days_Held</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -1819,12 +2378,18 @@
       <c r="F2" t="n">
         <v>14</v>
       </c>
+      <c r="G2" t="n">
+        <v>9779.98</v>
+      </c>
       <c r="H2" t="n">
         <v>-2.501</v>
       </c>
       <c r="I2" t="n">
         <v>-2.801</v>
       </c>
+      <c r="J2" t="n">
+        <v>-273.94</v>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>STOP_LOSS</t>
@@ -1861,12 +2426,18 @@
       <c r="F3" t="n">
         <v>13</v>
       </c>
+      <c r="G3" t="n">
+        <v>9873.76</v>
+      </c>
       <c r="H3" t="n">
         <v>0.241</v>
       </c>
       <c r="I3" t="n">
         <v>-0.059</v>
       </c>
+      <c r="J3" t="n">
+        <v>-5.83</v>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
           <t>TIME_EXIT</t>
@@ -1903,12 +2474,18 @@
       <c r="F4" t="n">
         <v>23</v>
       </c>
+      <c r="G4" t="n">
+        <v>9778.91</v>
+      </c>
       <c r="H4" t="n">
         <v>-1.216</v>
       </c>
       <c r="I4" t="n">
         <v>-1.516</v>
       </c>
+      <c r="J4" t="n">
+        <v>-148.25</v>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
           <t>TIME_EXIT</t>
@@ -1945,12 +2522,18 @@
       <c r="F5" t="n">
         <v>26</v>
       </c>
+      <c r="G5" t="n">
+        <v>9999.6</v>
+      </c>
       <c r="H5" t="n">
         <v>-1.092</v>
       </c>
       <c r="I5" t="n">
         <v>-1.392</v>
       </c>
+      <c r="J5" t="n">
+        <v>-139.19</v>
+      </c>
       <c r="K5" t="inlineStr">
         <is>
           <t>TIME_EXIT</t>
@@ -1987,12 +2570,18 @@
       <c r="F6" t="n">
         <v>7</v>
       </c>
+      <c r="G6" t="n">
+        <v>8857.1</v>
+      </c>
       <c r="H6" t="n">
         <v>-0.419</v>
       </c>
       <c r="I6" t="n">
         <v>-0.719</v>
       </c>
+      <c r="J6" t="n">
+        <v>-63.68</v>
+      </c>
       <c r="K6" t="inlineStr">
         <is>
           <t>TIME_EXIT</t>
@@ -2029,12 +2618,18 @@
       <c r="F7" t="n">
         <v>6</v>
       </c>
+      <c r="G7" t="n">
+        <v>8664.9</v>
+      </c>
       <c r="H7" t="n">
         <v>-2.5</v>
       </c>
       <c r="I7" t="n">
         <v>-2.8</v>
       </c>
+      <c r="J7" t="n">
+        <v>-242.62</v>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>STOP_LOSS</t>
@@ -2071,12 +2666,18 @@
       <c r="F8" t="n">
         <v>54</v>
       </c>
+      <c r="G8" t="n">
+        <v>9936.540000000001</v>
+      </c>
       <c r="H8" t="n">
         <v>-2.5</v>
       </c>
       <c r="I8" t="n">
         <v>-2.8</v>
       </c>
+      <c r="J8" t="n">
+        <v>-278.22</v>
+      </c>
       <c r="K8" t="inlineStr">
         <is>
           <t>STOP_LOSS</t>
@@ -2113,12 +2714,18 @@
       <c r="F9" t="n">
         <v>14</v>
       </c>
+      <c r="G9" t="n">
+        <v>9860.48</v>
+      </c>
       <c r="H9" t="n">
         <v>1.138</v>
       </c>
       <c r="I9" t="n">
         <v>0.838</v>
       </c>
+      <c r="J9" t="n">
+        <v>82.63</v>
+      </c>
       <c r="K9" t="inlineStr">
         <is>
           <t>TIME_EXIT</t>
@@ -2155,12 +2762,18 @@
       <c r="F10" t="n">
         <v>1</v>
       </c>
+      <c r="G10" t="n">
+        <v>33053.44</v>
+      </c>
       <c r="H10" t="n">
         <v>0.791</v>
       </c>
       <c r="I10" t="n">
         <v>0.491</v>
       </c>
+      <c r="J10" t="n">
+        <v>162.29</v>
+      </c>
       <c r="K10" t="inlineStr">
         <is>
           <t>TIME_EXIT</t>
@@ -2197,12 +2810,18 @@
       <c r="F11" t="n">
         <v>7</v>
       </c>
+      <c r="G11" t="n">
+        <v>9580.620000000001</v>
+      </c>
       <c r="H11" t="n">
         <v>1.621</v>
       </c>
       <c r="I11" t="n">
         <v>1.321</v>
       </c>
+      <c r="J11" t="n">
+        <v>126.56</v>
+      </c>
       <c r="K11" t="inlineStr">
         <is>
           <t>TIME_EXIT</t>
@@ -2239,12 +2858,18 @@
       <c r="F12" t="n">
         <v>16</v>
       </c>
+      <c r="G12" t="n">
+        <v>9455.68</v>
+      </c>
       <c r="H12" t="n">
         <v>-0.335</v>
       </c>
       <c r="I12" t="n">
         <v>-0.635</v>
       </c>
+      <c r="J12" t="n">
+        <v>-60.04</v>
+      </c>
       <c r="K12" t="inlineStr">
         <is>
           <t>TIME_EXIT</t>
@@ -2281,12 +2906,18 @@
       <c r="F13" t="n">
         <v>35</v>
       </c>
+      <c r="G13" t="n">
+        <v>9732.1</v>
+      </c>
       <c r="H13" t="n">
         <v>1.334</v>
       </c>
       <c r="I13" t="n">
         <v>1.034</v>
       </c>
+      <c r="J13" t="n">
+        <v>100.63</v>
+      </c>
       <c r="K13" t="inlineStr">
         <is>
           <t>TIME_EXIT</t>
@@ -2323,12 +2954,18 @@
       <c r="F14" t="n">
         <v>1</v>
       </c>
+      <c r="G14" t="n">
+        <v>12838.46</v>
+      </c>
       <c r="H14" t="n">
         <v>0.082</v>
       </c>
       <c r="I14" t="n">
         <v>-0.218</v>
       </c>
+      <c r="J14" t="n">
+        <v>-27.99</v>
+      </c>
       <c r="K14" t="inlineStr">
         <is>
           <t>TIME_EXIT</t>
@@ -2365,12 +3002,18 @@
       <c r="F15" t="n">
         <v>41</v>
       </c>
+      <c r="G15" t="n">
+        <v>9857.219999999999</v>
+      </c>
       <c r="H15" t="n">
         <v>-0.437</v>
       </c>
       <c r="I15" t="n">
         <v>-0.737</v>
       </c>
+      <c r="J15" t="n">
+        <v>-72.65000000000001</v>
+      </c>
       <c r="K15" t="inlineStr">
         <is>
           <t>TIME_EXIT</t>
@@ -2407,12 +3050,18 @@
       <c r="F16" t="n">
         <v>1</v>
       </c>
+      <c r="G16" t="n">
+        <v>5305.22</v>
+      </c>
       <c r="H16" t="n">
         <v>-2.5</v>
       </c>
       <c r="I16" t="n">
         <v>-2.8</v>
       </c>
+      <c r="J16" t="n">
+        <v>-148.55</v>
+      </c>
       <c r="K16" t="inlineStr">
         <is>
           <t>STOP_LOSS</t>
@@ -2449,12 +3098,18 @@
       <c r="F17" t="n">
         <v>1</v>
       </c>
+      <c r="G17" t="n">
+        <v>8824.34</v>
+      </c>
       <c r="H17" t="n">
         <v>-0.23</v>
       </c>
       <c r="I17" t="n">
         <v>-0.53</v>
       </c>
+      <c r="J17" t="n">
+        <v>-46.77</v>
+      </c>
       <c r="K17" t="inlineStr">
         <is>
           <t>TIME_EXIT</t>
@@ -2491,11 +3146,17 @@
       <c r="F18" t="n">
         <v>3</v>
       </c>
+      <c r="G18" t="n">
+        <v>7923</v>
+      </c>
       <c r="H18" t="n">
         <v>-0.417</v>
       </c>
       <c r="I18" t="n">
         <v>-0.717</v>
+      </c>
+      <c r="J18" t="n">
+        <v>-56.81</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -2523,57 +3184,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Order_ID</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Side</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Expected_Price</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Fill_Price</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Slippage</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -7578,27 +8239,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
@@ -7642,51 +8303,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cash_Available</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Invested_Capital</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Total_Equity</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Realized_PnL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Win_Rate_Pct</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Total_Trades</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Open_Positions</t>
         </is>
@@ -7755,6 +8416,39 @@
         <v>17</v>
       </c>
       <c r="I3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>12:57:48</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>198821.93</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>198821.93</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-1092.43</v>
+      </c>
+      <c r="G4" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="H4" t="n">
+        <v>17</v>
+      </c>
+      <c r="I4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>